<commit_message>
Align tracker with Port Department internship focus
</commit_message>
<xml_diff>
--- a/outputs/legislative_tracker_output.xlsx
+++ b/outputs/legislative_tracker_output.xlsx
@@ -12,9 +12,9 @@
     <sheet name="Summary Metrics" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Raw Data'!$A$1:$L$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Raw Data'!$A$1:$L$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'High Priority Bills'!$A$1:$L$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Summary Metrics'!$A$1:$E$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Summary Metrics'!$A$1:$E$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -51,7 +51,7 @@
       <color rgb="00000000"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -71,11 +71,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F6B26B"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00B6D7A8"/>
       </patternFill>
     </fill>
   </fills>
@@ -102,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -120,9 +115,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -225,8 +217,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RawDataTable" displayName="RawDataTable" ref="A1:L23" headerRowCount="1">
-  <autoFilter ref="A1:L23"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RawDataTable" displayName="RawDataTable" ref="A1:L18" headerRowCount="1">
+  <autoFilter ref="A1:L18"/>
   <tableColumns count="12">
     <tableColumn id="1" name="priority"/>
     <tableColumn id="2" name="relevance_score"/>
@@ -555,7 +547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L23"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1139,22 +1131,22 @@
       </c>
     </row>
     <row r="11" ht="54" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>LOW PRIORITY</t>
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>MEDIUM PRIORITY</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>35</v>
+        <v>65</v>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>H.R.4577</t>
+          <t>H. Rept. 119-212</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Defending American Property Abroad Act of 2025</t>
+          <t>FY2026 Transportation HUD Appropriations - Port Infrastructure Development Program</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1164,12 +1156,12 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Foreign Affairs</t>
+          <t>Appropriations</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Introduced</t>
+          <t>Reported</t>
         </is>
       </c>
       <c r="H11" s="4" t="n">
@@ -1180,73 +1172,73 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>Defines relevant port infrastructure including docks, piers, roads, storage structures, and port administration/security facilities. Potential relevance to international port access, cargo restrictions, and supply chain risk.</t>
+          <t>Committee report includes FY2026 Port Infrastructure Development Program funding recommendations and describes eligibility for port authorities, states, local governments, and transportation entities.</t>
         </is>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>port, harbor, marine terminal, freight, supply chain, security</t>
+          <t>appropriations, PIDP, port, infrastructure funding, cargo</t>
         </is>
       </c>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t>https://www.congress.gov/bill/119th-congress/house-bill/4577/text</t>
+          <t>https://www.congress.gov/committee-report/119th-congress/house-report/212/1</t>
         </is>
       </c>
     </row>
     <row r="12" ht="54" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>MEDIUM PRIORITY</t>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>HIGH PRIORITY</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>65</v>
+        <v>90</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>H. Rept. 119-212</t>
+          <t>NY S10222</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>FY2026 Transportation HUD Appropriations - Port Infrastructure Development Program</t>
+          <t>Relates to the organization of the Port Authority</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>U.S. House</t>
+          <t>New York Senate</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Appropriations</t>
+          <t>Corporations, Authorities And Commissions</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>Reported</t>
+          <t>In Committee</t>
         </is>
       </c>
       <c r="H12" s="4" t="n">
-        <v>45859</v>
+        <v>46149</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>302</v>
+        <v>12</v>
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>Committee report includes FY2026 Port Infrastructure Development Program funding recommendations and describes eligibility for port authorities, states, local governments, and transportation entities.</t>
+          <t>Active NY bill on Port Authority organization, appearance, notice, non-voting commissioners, capital planning, public hearings, and a Port Authority Transportation Advisory Committee.</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>appropriations, PIDP, port, infrastructure funding, cargo</t>
+          <t>New York, New Jersey, PANYNJ, port authority, capital plan, governance, transportation</t>
         </is>
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>https://www.congress.gov/committee-report/119th-congress/house-report/212/1</t>
+          <t>https://www.nysenate.gov/legislation/bills/2025/S10222</t>
         </is>
       </c>
     </row>
@@ -1261,7 +1253,7 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>NY S10222</t>
+          <t>NY A11291</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
@@ -1271,7 +1263,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>New York Senate</t>
+          <t>New York Assembly</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -1285,44 +1277,44 @@
         </is>
       </c>
       <c r="H13" s="4" t="n">
-        <v>46149</v>
+        <v>46157</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>Active NY bill on Port Authority organization, appearance, notice, non-voting commissioners, capital planning, public hearings, and a Port Authority Transportation Advisory Committee.</t>
+          <t>Assembly companion associated with NY S10222 addressing Port Authority organization, notice, capital planning, and bi-state oversight. Important for governance and planning workflows.</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>New York, New Jersey, PANYNJ, port authority, capital plan, governance, transportation</t>
+          <t>New York, New Jersey, PANYNJ, port authority, capital plan, governance</t>
         </is>
       </c>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>https://www.nysenate.gov/legislation/bills/2025/S10222</t>
+          <t>https://legislation.nysenate.gov/pdf/bills/2025/A11291</t>
         </is>
       </c>
     </row>
     <row r="14" ht="54" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>HIGH PRIORITY</t>
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>MEDIUM PRIORITY</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>NY A11291</t>
+          <t>NY A10056</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Relates to the organization of the Port Authority</t>
+          <t>Relates to Port Authority organization, appearance and notice</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1341,14 +1333,14 @@
         </is>
       </c>
       <c r="H14" s="4" t="n">
-        <v>46157</v>
+        <v>46052</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>4</v>
+        <v>109</v>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>Assembly companion associated with NY S10222 addressing Port Authority organization, notice, capital planning, and bi-state oversight. Important for governance and planning workflows.</t>
+          <t>Active Assembly bill amending the Port Authority compact laws in relation to organization, appearance, notice, commissioner qualifications, and capital plan requirements.</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
@@ -1358,7 +1350,7 @@
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>https://legislation.nysenate.gov/pdf/bills/2025/A11291</t>
+          <t>https://www.nysenate.gov/legislation/bills/2025/A10056</t>
         </is>
       </c>
     </row>
@@ -1373,17 +1365,17 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>NY A10056</t>
+          <t>NY S6939</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Relates to Port Authority organization, appearance and notice</t>
+          <t>Collective employment negotiations, debt notice, and capital plans at PANYNJ</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>New York Assembly</t>
+          <t>New York Senate</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -1397,24 +1389,24 @@
         </is>
       </c>
       <c r="H15" s="4" t="n">
-        <v>46052</v>
+        <v>46029</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>Active Assembly bill amending the Port Authority compact laws in relation to organization, appearance, notice, commissioner qualifications, and capital plan requirements.</t>
+          <t>Active NY bill requiring Port Authority legislative appearances, debt issuance notice, capital plan transparency, capital status hearings, and collective negotiation protections.</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>New York, New Jersey, PANYNJ, port authority, capital plan, governance</t>
+          <t>New York, New Jersey, PANYNJ, port authority, capital plan, labor, debt</t>
         </is>
       </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t>https://www.nysenate.gov/legislation/bills/2025/A10056</t>
+          <t>https://www.nysenate.gov/legislation/bills/2025/S6939</t>
         </is>
       </c>
     </row>
@@ -1429,124 +1421,124 @@
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>NY S6939</t>
+          <t>NJ S289</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Collective employment negotiations, debt notice, and capital plans at PANYNJ</t>
+          <t>Port Authority of New York and New Jersey Cargo Facility Charge Act</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>New York Senate</t>
+          <t>New Jersey Senate</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Corporations, Authorities And Commissions</t>
+          <t>Transportation</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>In Committee</t>
+          <t>Introduced</t>
         </is>
       </c>
       <c r="H16" s="4" t="n">
-        <v>46029</v>
+        <v>43844</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>132</v>
+        <v>2317</v>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>Active NY bill requiring Port Authority legislative appearances, debt issuance notice, capital plan transparency, capital status hearings, and collective negotiation protections.</t>
+          <t>Establishes a Port Authority cargo facility charge framework for export and import cargo handled through PANYNJ-related facilities. Older but operationally relevant for cargo cost and facility policy monitoring.</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>New York, New Jersey, PANYNJ, port authority, capital plan, labor, debt</t>
+          <t>New Jersey, PANYNJ, cargo, freight, port, facility charge</t>
         </is>
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>https://www.nysenate.gov/legislation/bills/2025/S6939</t>
+          <t>https://pub.njleg.state.nj.us/Bills/2020/S0500/289_I1.HTM</t>
         </is>
       </c>
     </row>
     <row r="17" ht="54" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>LOW PRIORITY</t>
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>MEDIUM PRIORITY</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>NY A8889</t>
+          <t>NJ S4670</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Customer Savings and Reliability Act</t>
+          <t>Delaware River and Bay of New Jersey Authority and marine transportation updates</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>New York Assembly</t>
+          <t>New Jersey Senate</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Corporations, Authorities And Commissions</t>
+          <t>Transportation</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>In Committee</t>
+          <t>Introduced</t>
         </is>
       </c>
       <c r="H17" s="4" t="n">
-        <v>46029</v>
+        <v>45838</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>132</v>
+        <v>323</v>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>Active NY utility transition bill with critical infrastructure and regional planning implications. Included as a lower-priority watch item because energy transition planning can affect large infrastructure operators.</t>
+          <t>New Jersey measure touching marine terminals, port facilities, commerce facilities, maritime industry, navigation channels, and the Marine Transportation System. Relevant as a statewide maritime infrastructure watch item.</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>New York, infrastructure, critical infrastructure, energy transition, workforce</t>
+          <t>New Jersey, maritime, marine terminal, port facilities, navigation, infrastructure</t>
         </is>
       </c>
       <c r="L17" s="5" t="inlineStr">
         <is>
-          <t>https://www.nysenate.gov/legislation/bills/2025/A8889</t>
+          <t>https://pub.njleg.state.nj.us/Bills/2024/S5000/4670_I1.HTM</t>
         </is>
       </c>
     </row>
     <row r="18" ht="54" customHeight="1">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>MEDIUM PRIORITY</t>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>HIGH PRIORITY</t>
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>NJ S2098</t>
+          <t>NJ S3748</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>PANYNJ restrictions on employment, gifts, compensation, and tuition reimbursement</t>
+          <t>South Jersey Transportation Authority membership and transportation scope</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1556,319 +1548,39 @@
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>State Government</t>
+          <t>Transportation</t>
         </is>
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>Prefiled / Introduced Pending Technical Review</t>
+          <t>Introduced</t>
         </is>
       </c>
       <c r="H18" s="4" t="n">
-        <v>46035</v>
+        <v>46097</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>126</v>
+        <v>64</v>
       </c>
       <c r="J18" s="3" t="inlineStr">
         <is>
-          <t>New Jersey bill imposing restrictions on Port Authority commissioners, officers, and employees regarding travel, compensation, gifts, outside employment, toll/fare reimbursements, and tuition reimbursement.</t>
+          <t>Adds Burlington County to SJTA and references regional transportation facilities including air freight and marine passenger infrastructure. Relevant for broader NJ transportation planning context.</t>
         </is>
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>New Jersey, PANYNJ, port authority, governance, workforce, compensation</t>
+          <t>New Jersey, transportation, air freight, marine, infrastructure</t>
         </is>
       </c>
       <c r="L18" s="5" t="inlineStr">
         <is>
-          <t>https://pub.njleg.state.nj.us/Bills/2026/S2500/2098_I1.PDF</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="54" customHeight="1">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>MEDIUM PRIORITY</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="n">
-        <v>70</v>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>NJ A688</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>E-ZPass toll deduction for certain tolls paid</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>New Jersey Assembly</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr">
-        <is>
-          <t>Transportation and Independent Authorities</t>
-        </is>
-      </c>
-      <c r="G19" s="3" t="inlineStr">
-        <is>
-          <t>Prefiled / Introduced Pending Technical Review</t>
-        </is>
-      </c>
-      <c r="H19" s="4" t="n">
-        <v>46035</v>
-      </c>
-      <c r="I19" s="3" t="n">
-        <v>126</v>
-      </c>
-      <c r="J19" s="3" t="inlineStr">
-        <is>
-          <t>New Jersey bill providing a gross income tax deduction for certain E-ZPass tolls paid on toll roadways and interstate bridges/tunnels, including facilities operated by the Port Authority of New York and New Jersey.</t>
-        </is>
-      </c>
-      <c r="K19" s="3" t="inlineStr">
-        <is>
-          <t>New Jersey, PANYNJ, toll, bridge, tunnel, transportation</t>
-        </is>
-      </c>
-      <c r="L19" s="5" t="inlineStr">
-        <is>
-          <t>https://pub.njleg.state.nj.us/Bills/2026/A1000/688_I1.HTM</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="54" customHeight="1">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>MEDIUM PRIORITY</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="n">
-        <v>70</v>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>NJ S289</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>Port Authority of New York and New Jersey Cargo Facility Charge Act</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>New Jersey Senate</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>Transportation</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>Introduced</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="n">
-        <v>43844</v>
-      </c>
-      <c r="I20" s="3" t="n">
-        <v>2317</v>
-      </c>
-      <c r="J20" s="3" t="inlineStr">
-        <is>
-          <t>Establishes a Port Authority cargo facility charge framework for export and import cargo handled through PANYNJ-related facilities. Older but operationally relevant for cargo cost and facility policy monitoring.</t>
-        </is>
-      </c>
-      <c r="K20" s="3" t="inlineStr">
-        <is>
-          <t>New Jersey, PANYNJ, cargo, freight, port, facility charge</t>
-        </is>
-      </c>
-      <c r="L20" s="5" t="inlineStr">
-        <is>
-          <t>https://pub.njleg.state.nj.us/Bills/2020/S0500/289_I1.HTM</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="54" customHeight="1">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>MEDIUM PRIORITY</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="n">
-        <v>70</v>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>NJ S4670</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>Delaware River and Bay of New Jersey Authority and marine transportation updates</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>New Jersey Senate</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>Transportation</t>
-        </is>
-      </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>Introduced</t>
-        </is>
-      </c>
-      <c r="H21" s="4" t="n">
-        <v>45838</v>
-      </c>
-      <c r="I21" s="3" t="n">
-        <v>323</v>
-      </c>
-      <c r="J21" s="3" t="inlineStr">
-        <is>
-          <t>New Jersey measure touching marine terminals, port facilities, commerce facilities, maritime industry, navigation channels, and the Marine Transportation System. Relevant as a statewide maritime infrastructure watch item.</t>
-        </is>
-      </c>
-      <c r="K21" s="3" t="inlineStr">
-        <is>
-          <t>New Jersey, maritime, marine terminal, port facilities, navigation, infrastructure</t>
-        </is>
-      </c>
-      <c r="L21" s="5" t="inlineStr">
-        <is>
-          <t>https://pub.njleg.state.nj.us/Bills/2024/S5000/4670_I1.HTM</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="54" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>HIGH PRIORITY</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="n">
-        <v>90</v>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>NJ S3748</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>South Jersey Transportation Authority membership and transportation scope</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>New Jersey Senate</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>Transportation</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>Introduced</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="n">
-        <v>46097</v>
-      </c>
-      <c r="I22" s="3" t="n">
-        <v>64</v>
-      </c>
-      <c r="J22" s="3" t="inlineStr">
-        <is>
-          <t>Adds Burlington County to SJTA and references regional transportation facilities including air freight and marine passenger infrastructure. Relevant for broader NJ transportation planning context.</t>
-        </is>
-      </c>
-      <c r="K22" s="3" t="inlineStr">
-        <is>
-          <t>New Jersey, transportation, air freight, marine, infrastructure</t>
-        </is>
-      </c>
-      <c r="L22" s="5" t="inlineStr">
-        <is>
           <t>https://pub.njleg.state.nj.us/Bills/2026/S4000/3748_I1.HTM</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="54" customHeight="1">
-      <c r="A23" s="7" t="inlineStr">
-        <is>
-          <t>LOW PRIORITY</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>NJ S1401</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="inlineStr">
-        <is>
-          <t>Public employee retirement system provisions including South Jersey Port employees</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>New Jersey Senate</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
-        <is>
-          <t>State Government</t>
-        </is>
-      </c>
-      <c r="G23" s="3" t="inlineStr">
-        <is>
-          <t>Introduced</t>
-        </is>
-      </c>
-      <c r="H23" s="4" t="n">
-        <v>45300</v>
-      </c>
-      <c r="I23" s="3" t="n">
-        <v>861</v>
-      </c>
-      <c r="J23" s="3" t="inlineStr">
-        <is>
-          <t>Includes provisions related to South Jersey Port Corporation employees and related Delaware River Port Authority entities. Included as a workforce and public employment watch item.</t>
-        </is>
-      </c>
-      <c r="K23" s="3" t="inlineStr">
-        <is>
-          <t>New Jersey, South Jersey Port, workforce, public employees, port authority</t>
-        </is>
-      </c>
-      <c r="L23" s="5" t="inlineStr">
-        <is>
-          <t>https://pub.njleg.state.nj.us/Bills/2024/S1500/1401_I1.HTM</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L23"/>
-  <conditionalFormatting sqref="B2:B23">
+  <autoFilter ref="A1:L18"/>
+  <conditionalFormatting sqref="B2:B18">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
       <formula>80</formula>
     </cfRule>
@@ -1898,15 +1610,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId23"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId18"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2253,7 +1960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2297,7 +2004,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="C2" s="3" t="inlineStr"/>
       <c r="D2" s="3" t="inlineStr"/>
@@ -2323,7 +2030,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C4" s="3" t="inlineStr"/>
       <c r="D4" s="3" t="inlineStr"/>
@@ -2336,7 +2043,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
       <c r="D5" s="3" t="inlineStr"/>
@@ -2349,7 +2056,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>63.86</v>
+        <v>69.41</v>
       </c>
       <c r="C6" s="3" t="inlineStr"/>
       <c r="D6" s="3" t="inlineStr"/>
@@ -2401,10 +2108,10 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>73</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" ht="12" customHeight="1">
@@ -2427,14 +2134,14 @@
       <c r="B12" s="3" t="inlineStr"/>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Foreign Affairs</t>
+          <t>House Transportation and Infrastructure; Senate Commerce</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>35</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13" ht="12" customHeight="1">
@@ -2442,14 +2149,14 @@
       <c r="B13" s="3" t="inlineStr"/>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>House Transportation and Infrastructure; Senate Commerce</t>
+          <t>Transportation</t>
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>80</v>
+        <v>76.67</v>
       </c>
     </row>
     <row r="14" ht="12" customHeight="1">
@@ -2457,14 +2164,14 @@
       <c r="B14" s="3" t="inlineStr"/>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>State Government</t>
+          <t>Transportation and Infrastructure</t>
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>37.5</v>
+        <v>60</v>
       </c>
     </row>
     <row r="15" ht="12" customHeight="1">
@@ -2472,63 +2179,18 @@
       <c r="B15" s="3" t="inlineStr"/>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Transportation</t>
+          <t>Transportation and Infrastructure; Environment and Public Works</t>
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>76.67</v>
-      </c>
-    </row>
-    <row r="16" ht="12" customHeight="1">
-      <c r="A16" s="3" t="inlineStr"/>
-      <c r="B16" s="3" t="inlineStr"/>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>Transportation and Independent Authorities</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="3" t="n">
         <v>70</v>
       </c>
     </row>
-    <row r="17" ht="12" customHeight="1">
-      <c r="A17" s="3" t="inlineStr"/>
-      <c r="B17" s="3" t="inlineStr"/>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>Transportation and Infrastructure</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E17" s="3" t="n">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="18" ht="12" customHeight="1">
-      <c r="A18" s="3" t="inlineStr"/>
-      <c r="B18" s="3" t="inlineStr"/>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Transportation and Infrastructure; Environment and Public Works</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E18" s="3" t="n">
-        <v>70</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:E18"/>
+  <autoFilter ref="A1:E15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Finalize formal multi-level legislative tracker
</commit_message>
<xml_diff>
--- a/outputs/legislative_tracker_output.xlsx
+++ b/outputs/legislative_tracker_output.xlsx
@@ -12,9 +12,9 @@
     <sheet name="Summary Metrics" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Raw Data'!$A$1:$L$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'High Priority Bills'!$A$1:$L$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Summary Metrics'!$A$1:$E$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Raw Data'!$A$1:$L$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'High Priority Bills'!$A$1:$L$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Summary Metrics'!$A$1:$E$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -51,7 +51,7 @@
       <color rgb="00000000"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -71,6 +71,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F6B26B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B6D7A8"/>
       </patternFill>
     </fill>
   </fills>
@@ -97,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -115,6 +120,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -217,8 +225,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RawDataTable" displayName="RawDataTable" ref="A1:L18" headerRowCount="1">
-  <autoFilter ref="A1:L18"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RawDataTable" displayName="RawDataTable" ref="A1:L37" headerRowCount="1">
+  <autoFilter ref="A1:L37"/>
   <tableColumns count="12">
     <tableColumn id="1" name="priority"/>
     <tableColumn id="2" name="relevance_score"/>
@@ -238,8 +246,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="HighPriorityBillsTable" displayName="HighPriorityBillsTable" ref="A1:L5" headerRowCount="1">
-  <autoFilter ref="A1:L5"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="HighPriorityBillsTable" displayName="HighPriorityBillsTable" ref="A1:L11" headerRowCount="1">
+  <autoFilter ref="A1:L11"/>
   <tableColumns count="12">
     <tableColumn id="1" name="priority"/>
     <tableColumn id="2" name="relevance_score"/>
@@ -547,7 +555,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -664,7 +672,7 @@
         <v>45818</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
@@ -720,7 +728,7 @@
         <v>45748</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
@@ -776,7 +784,7 @@
         <v>46055</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
@@ -832,7 +840,7 @@
         <v>46008</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
@@ -888,7 +896,7 @@
         <v>45925</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
@@ -944,7 +952,7 @@
         <v>45777</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
@@ -1000,7 +1008,7 @@
         <v>45778</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
@@ -1056,7 +1064,7 @@
         <v>45813</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
@@ -1112,7 +1120,7 @@
         <v>45847</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
@@ -1168,7 +1176,7 @@
         <v>45859</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
@@ -1187,114 +1195,114 @@
       </c>
     </row>
     <row r="12" ht="54" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>HIGH PRIORITY</t>
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>MEDIUM PRIORITY</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>90</v>
+        <v>55</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>NY S10222</t>
+          <t>S.2465</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Relates to the organization of the Port Authority</t>
+          <t>FY2026 Transportation HUD Appropriations Act</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>New York Senate</t>
+          <t>U.S. Senate</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>Corporations, Authorities And Commissions</t>
+          <t>Appropriations</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>In Committee</t>
+          <t>Introduced</t>
         </is>
       </c>
       <c r="H12" s="4" t="n">
-        <v>46149</v>
+        <v>45862</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>12</v>
+        <v>300</v>
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>Active NY bill on Port Authority organization, appearance, notice, non-voting commissioners, capital planning, public hearings, and a Port Authority Transportation Advisory Committee.</t>
+          <t>Senate FY2026 transportation appropriations bill with MARAD, America's Marine Highway, state maritime academy, small shipyard, and Port Infrastructure Development Program funding language. Relevant to federal port grants, maritime workforce, and goods movement funding.</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>New York, New Jersey, PANYNJ, port authority, capital plan, governance, transportation</t>
+          <t>appropriations, port infrastructure development program, MARAD, maritime workforce, marine highway, infrastructure</t>
         </is>
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>https://www.nysenate.gov/legislation/bills/2025/S10222</t>
+          <t>https://www.congress.gov/bill/119th-congress/senate-bill/2465</t>
         </is>
       </c>
     </row>
     <row r="13" ht="54" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>HIGH PRIORITY</t>
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>MEDIUM PRIORITY</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>90</v>
+        <v>65</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>NY A11291</t>
+          <t>S. Rept. 119-47</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Relates to the organization of the Port Authority</t>
+          <t>FY2026 Transportation HUD Appropriations Senate Report</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>New York Assembly</t>
+          <t>U.S. Senate</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>Corporations, Authorities And Commissions</t>
+          <t>Appropriations</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>In Committee</t>
+          <t>Reported</t>
         </is>
       </c>
       <c r="H13" s="4" t="n">
-        <v>46157</v>
+        <v>45862</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>4</v>
+        <v>300</v>
       </c>
       <c r="J13" s="3" t="inlineStr">
         <is>
-          <t>Assembly companion associated with NY S10222 addressing Port Authority organization, notice, capital planning, and bi-state oversight. Important for governance and planning workflows.</t>
+          <t>Senate appropriations report covering FY2026 transportation funding, including Maritime Administration and Port Infrastructure Development Program recommendations. Relevant to tracking federal funding direction for port capital planning.</t>
         </is>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>New York, New Jersey, PANYNJ, port authority, capital plan, governance</t>
+          <t>appropriations, port infrastructure development program, MARAD, transportation funding, infrastructure</t>
         </is>
       </c>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>https://legislation.nysenate.gov/pdf/bills/2025/A11291</t>
+          <t>https://www.congress.gov/committee-report/119th-congress/senate-report/47</t>
         </is>
       </c>
     </row>
@@ -1305,108 +1313,108 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>NY A10056</t>
+          <t>S.257</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Relates to Port Authority organization, appearance and notice</t>
+          <t>Promoting Resilient Supply Chains Act of 2025</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>New York Assembly</t>
+          <t>U.S. Senate / U.S. House</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Corporations, Authorities And Commissions</t>
+          <t>Commerce; Energy and Commerce</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>In Committee</t>
+          <t>Passed Senate</t>
         </is>
       </c>
       <c r="H14" s="4" t="n">
-        <v>46052</v>
+        <v>45841</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>109</v>
+        <v>321</v>
       </c>
       <c r="J14" s="3" t="inlineStr">
         <is>
-          <t>Active Assembly bill amending the Port Authority compact laws in relation to organization, appearance, notice, commissioner qualifications, and capital plan requirements.</t>
+          <t>Creates federal supply chain mapping, modeling, and resilience work. Relevant to port policy because disruptions in critical supply chains affect cargo flow, logistics networks, and regional freight planning.</t>
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>New York, New Jersey, PANYNJ, port authority, capital plan, governance</t>
+          <t>supply chain, logistics, freight, resilience, commerce</t>
         </is>
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>https://www.nysenate.gov/legislation/bills/2025/A10056</t>
+          <t>https://www.congress.gov/bill/119th-congress/senate-bill/257/all-info</t>
         </is>
       </c>
     </row>
     <row r="15" ht="54" customHeight="1">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>MEDIUM PRIORITY</t>
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>LOW PRIORITY</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>NY S6939</t>
+          <t>H.R.4183</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Collective employment negotiations, debt notice, and capital plans at PANYNJ</t>
+          <t>Federal Maritime Commission Reauthorization Act of 2025</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>New York Senate</t>
+          <t>U.S. House</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>Corporations, Authorities And Commissions</t>
+          <t>Transportation and Infrastructure</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>In Committee</t>
+          <t>Introduced</t>
         </is>
       </c>
       <c r="H15" s="4" t="n">
-        <v>46029</v>
+        <v>45834</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>132</v>
+        <v>328</v>
       </c>
       <c r="J15" s="3" t="inlineStr">
         <is>
-          <t>Active NY bill requiring Port Authority legislative appearances, debt issuance notice, capital plan transparency, capital status hearings, and collective negotiation protections.</t>
+          <t>Reauthorizes the Federal Maritime Commission for fiscal years 2026 through 2029. Relevant to ocean shipping, carrier oversight, maritime commerce, and policy issues affecting port users.</t>
         </is>
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>New York, New Jersey, PANYNJ, port authority, capital plan, labor, debt</t>
+          <t>maritime, shipping, supply chain, federal authorization, port</t>
         </is>
       </c>
       <c r="L15" s="5" t="inlineStr">
         <is>
-          <t>https://www.nysenate.gov/legislation/bills/2025/S6939</t>
+          <t>https://www.congress.gov/bill/119th-congress/house-bill/4183/history</t>
         </is>
       </c>
     </row>
@@ -1417,26 +1425,26 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>NJ S289</t>
+          <t>H.R.971</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Port Authority of New York and New Jersey Cargo Facility Charge Act</t>
+          <t>RAIL Act</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>New Jersey Senate</t>
+          <t>U.S. House</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Transportation</t>
+          <t>Transportation and Infrastructure</t>
         </is>
       </c>
       <c r="G16" s="3" t="inlineStr">
@@ -1445,80 +1453,80 @@
         </is>
       </c>
       <c r="H16" s="4" t="n">
-        <v>43844</v>
+        <v>45692</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>2317</v>
+        <v>470</v>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>Establishes a Port Authority cargo facility charge framework for export and import cargo handled through PANYNJ-related facilities. Older but operationally relevant for cargo cost and facility policy monitoring.</t>
+          <t>Rail infrastructure and safety measure referred to the House rail subcommittee. Relevant as a watch item because port competitiveness depends on inland freight rail capacity, safety, and intermodal connections.</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>New Jersey, PANYNJ, cargo, freight, port, facility charge</t>
+          <t>freight rail, rail, intermodal, infrastructure, logistics</t>
         </is>
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>https://pub.njleg.state.nj.us/Bills/2020/S0500/289_I1.HTM</t>
+          <t>https://www.congress.gov/index.php/bill/119th-congress/house-bill/971</t>
         </is>
       </c>
     </row>
     <row r="17" ht="54" customHeight="1">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>MEDIUM PRIORITY</t>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>HIGH PRIORITY</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>NJ S4670</t>
+          <t>NY S10222</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Delaware River and Bay of New Jersey Authority and marine transportation updates</t>
+          <t>Relates to the organization of the Port Authority</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>New Jersey Senate</t>
+          <t>New York Senate</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>Transportation</t>
+          <t>Corporations, Authorities And Commissions</t>
         </is>
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>Introduced</t>
+          <t>In Committee</t>
         </is>
       </c>
       <c r="H17" s="4" t="n">
-        <v>45838</v>
+        <v>46149</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>323</v>
+        <v>13</v>
       </c>
       <c r="J17" s="3" t="inlineStr">
         <is>
-          <t>New Jersey measure touching marine terminals, port facilities, commerce facilities, maritime industry, navigation channels, and the Marine Transportation System. Relevant as a statewide maritime infrastructure watch item.</t>
+          <t>Active NY bill on Port Authority organization, appearance, notice, non-voting commissioners, capital planning, public hearings, and a Port Authority Transportation Advisory Committee.</t>
         </is>
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>New Jersey, maritime, marine terminal, port facilities, navigation, infrastructure</t>
+          <t>New York, New Jersey, PANYNJ, port authority, capital plan, governance, transportation</t>
         </is>
       </c>
       <c r="L17" s="5" t="inlineStr">
         <is>
-          <t>https://pub.njleg.state.nj.us/Bills/2024/S5000/4670_I1.HTM</t>
+          <t>https://www.nysenate.gov/legislation/bills/2025/S10222</t>
         </is>
       </c>
     </row>
@@ -1533,54 +1541,1118 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
+          <t>NY A11291</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Relates to the organization of the Port Authority</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>New York Assembly</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>Corporations, Authorities And Commissions</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>In Committee</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="n">
+        <v>46157</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>Assembly companion associated with NY S10222 addressing Port Authority organization, notice, capital planning, and bi-state oversight. Important for governance and planning workflows.</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>New York, New Jersey, PANYNJ, port authority, capital plan, governance</t>
+        </is>
+      </c>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>https://www.nysenate.gov/legislation/bills/2025/A11291</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="54" customHeight="1">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>MEDIUM PRIORITY</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>NY A10056</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Relates to Port Authority organization, appearance and notice</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>New York Assembly</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Corporations, Authorities And Commissions</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>In Committee</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="n">
+        <v>46052</v>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>110</v>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>Active Assembly bill amending the Port Authority compact laws in relation to organization, appearance, notice, commissioner qualifications, and capital plan requirements.</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>New York, New Jersey, PANYNJ, port authority, capital plan, governance</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>https://www.nysenate.gov/legislation/bills/2025/A10056</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="54" customHeight="1">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>MEDIUM PRIORITY</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>NY S6939</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Collective employment negotiations, debt notice, and capital plans at PANYNJ</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>New York Senate</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Corporations, Authorities And Commissions</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>In Committee</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="n">
+        <v>46029</v>
+      </c>
+      <c r="I20" s="3" t="n">
+        <v>133</v>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>Active NY bill requiring Port Authority legislative appearances, debt issuance notice, capital plan transparency, capital status hearings, and collective negotiation protections.</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>New York, New Jersey, PANYNJ, port authority, capital plan, labor, debt</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>https://www.nysenate.gov/legislation/bills/2025/S6939</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="54" customHeight="1">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>MEDIUM PRIORITY</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>NJ S289</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Port Authority of New York and New Jersey Cargo Facility Charge Act</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey Senate</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>Introduced</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="n">
+        <v>43844</v>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>2318</v>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>Establishes a Port Authority cargo facility charge framework for export and import cargo handled through PANYNJ-related facilities. Older but operationally relevant for cargo cost and facility policy monitoring.</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey, PANYNJ, cargo, freight, port, facility charge</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>https://pub.njleg.state.nj.us/Bills/2020/S0500/289_I1.HTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="54" customHeight="1">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>MEDIUM PRIORITY</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>NJ S4670</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Delaware River and Bay of New Jersey Authority and marine transportation updates</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey Senate</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>Introduced</t>
+        </is>
+      </c>
+      <c r="H22" s="4" t="n">
+        <v>45838</v>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>324</v>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey measure touching marine terminals, port facilities, commerce facilities, maritime industry, navigation channels, and the Marine Transportation System. Relevant as a statewide maritime infrastructure watch item.</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey, maritime, marine terminal, port facilities, navigation, infrastructure</t>
+        </is>
+      </c>
+      <c r="L22" s="5" t="inlineStr">
+        <is>
+          <t>https://pub.njleg.state.nj.us/Bills/2024/S5000/4670_I1.HTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="54" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>HIGH PRIORITY</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
           <t>NJ S3748</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D23" s="3" t="inlineStr">
         <is>
           <t>South Jersey Transportation Authority membership and transportation scope</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>New Jersey Senate</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>Transportation</t>
         </is>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>Introduced</t>
         </is>
       </c>
-      <c r="H18" s="4" t="n">
+      <c r="H23" s="4" t="n">
         <v>46097</v>
       </c>
-      <c r="I18" s="3" t="n">
-        <v>64</v>
-      </c>
-      <c r="J18" s="3" t="inlineStr">
+      <c r="I23" s="3" t="n">
+        <v>65</v>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
         <is>
           <t>Adds Burlington County to SJTA and references regional transportation facilities including air freight and marine passenger infrastructure. Relevant for broader NJ transportation planning context.</t>
         </is>
       </c>
-      <c r="K18" s="3" t="inlineStr">
+      <c r="K23" s="3" t="inlineStr">
         <is>
           <t>New Jersey, transportation, air freight, marine, infrastructure</t>
         </is>
       </c>
-      <c r="L18" s="5" t="inlineStr">
+      <c r="L23" s="5" t="inlineStr">
         <is>
           <t>https://pub.njleg.state.nj.us/Bills/2026/S4000/3748_I1.HTM</t>
         </is>
       </c>
     </row>
+    <row r="24" ht="54" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>HIGH PRIORITY</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>NJ A4236</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>High-growth STEM and transportation logistics workforce update</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey Assembly</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Labor</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Introduced</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="n">
+        <v>46076</v>
+      </c>
+      <c r="I24" s="3" t="n">
+        <v>86</v>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>Updates high-growth industry and workforce language including transportation, logistics, and distribution. Relevant to workforce pathways that support port, freight, warehousing, and supply chain employers.</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey, workforce development, transportation, logistics, distribution</t>
+        </is>
+      </c>
+      <c r="L24" s="5" t="inlineStr">
+        <is>
+          <t>https://pub.njleg.state.nj.us/Bills/2026/A4500/4236_I1.HTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="54" customHeight="1">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>MEDIUM PRIORITY</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>NJ S1498</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey Pathways to Career Opportunities Initiative Act</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey Senate</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>Labor</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Introduced</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="n">
+        <v>46035</v>
+      </c>
+      <c r="I25" s="3" t="n">
+        <v>127</v>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>Codifies career pathway and workforce innovation initiatives through county colleges and employer partnerships. Relevant to transportation, logistics, distribution, and port-adjacent workforce development.</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey, workforce development, career pathways, logistics, distribution</t>
+        </is>
+      </c>
+      <c r="L25" s="5" t="inlineStr">
+        <is>
+          <t>https://pub.njleg.state.nj.us/Bills/2026/S1500/1498_I1.HTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="54" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>HIGH PRIORITY</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>NJ S3593</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey Works Act pre-employment and work readiness training</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey Senate</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Labor</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Reported Committee</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="n">
+        <v>46083</v>
+      </c>
+      <c r="I26" s="3" t="n">
+        <v>79</v>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>Provides tax credits for approved pre-employment and work readiness training programs for in-demand jobs. Relevant to building workforce pipelines for logistics, port operations, and regional goods movement employers.</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey, workforce development, work readiness, logistics, training</t>
+        </is>
+      </c>
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>https://pub.njleg.state.nj.us/Bills/2026/S4000/3593_S1.HTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="54" customHeight="1">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>MEDIUM PRIORITY</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>NJ A4740</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Safe Commercial Routes Act - Commercial Driver Human Trafficking Awareness Training</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey Assembly</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>Introduced</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="n">
+        <v>46097</v>
+      </c>
+      <c r="I27" s="3" t="n">
+        <v>65</v>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>Requires commercial driver applicants and renewals to complete human trafficking awareness training. Relevant to commercial routes, logistics hubs, international shipping ports, truck stops, warehouses, and transportation safety.</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey, commercial routes, logistics hubs, trucking, transportation, ports</t>
+        </is>
+      </c>
+      <c r="L27" s="5" t="inlineStr">
+        <is>
+          <t>https://pub.njleg.state.nj.us/Bills/2026/A5000/4740_I1.HTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="54" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>HIGH PRIORITY</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>NJ S3695</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Transportation Authority of New Jersey governance and transfer act</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey Senate</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Introduced</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="n">
+        <v>46077</v>
+      </c>
+      <c r="I28" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>Creates a statewide transportation authority structure and transfers certain transportation entities while preserving rules, bonding powers, employees, and operational obligations. Relevant as a New Jersey transportation governance and infrastructure oversight watch item.</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey, transportation authority, infrastructure, governance, operations, workforce</t>
+        </is>
+      </c>
+      <c r="L28" s="5" t="inlineStr">
+        <is>
+          <t>https://pub.njleg.state.nj.us/Bills/2026/S4000/3695_I1.HTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="54" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>HIGH PRIORITY</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>NJ S3790</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Transportation authority reporting and Port Authority-related oversight</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey Senate</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>Introduced</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="n">
+        <v>46122</v>
+      </c>
+      <c r="I29" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>Requires reporting and oversight related to major transportation authorities and references the Port Authority of New York and New Jersey. Relevant to governance, accountability, workforce, and regional transportation policy monitoring.</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey, PANYNJ, Port Authority, transportation authority, oversight, workforce</t>
+        </is>
+      </c>
+      <c r="L29" s="5" t="inlineStr">
+        <is>
+          <t>https://pub.njleg.state.nj.us/Bills/2026/S4000/3790_I1.PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="54" customHeight="1">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>MEDIUM PRIORITY</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>65</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>NYC Int 0051-2026</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Feasibility study of zero-emission port operations</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>New York City Council</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>Committee on Transportation and Infrastructure</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>Referred to Committee</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="n">
+        <v>46051</v>
+      </c>
+      <c r="I30" s="3" t="n">
+        <v>111</v>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>Requires a feasibility study of zero-emission port operations, including shore power for commercial maritime vessels and incentives for low- or zero-emission vessels. Directly relevant to clean port planning and maritime emissions policy.</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>NYC, zero-emission port operations, shore power, maritime, clean ports</t>
+        </is>
+      </c>
+      <c r="L30" s="5" t="inlineStr">
+        <is>
+          <t>https://legistar.council.nyc.gov/LegislationDetail.aspx?GUID=C0FAF072-A278-41C2-9E72-06B6C54F48E1&amp;ID=7861419&amp;Options=&amp;Search=</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="54" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>LOW PRIORITY</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>NYC Int 0052-2026</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Green port water-dependent manufacturing and maritime industrial areas</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>New York City Council</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>Committee on Zoning and Franchises</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Referred to Committee</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="n">
+        <v>46051</v>
+      </c>
+      <c r="I31" s="3" t="n">
+        <v>111</v>
+      </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>Defines green port water-dependent manufacturing and significant maritime industrial areas. Relevant to waterfront land use, maritime industrial preservation, port-adjacent manufacturing, and zero-emission maritime economy planning.</t>
+        </is>
+      </c>
+      <c r="K31" s="3" t="inlineStr">
+        <is>
+          <t>NYC, green port, waterfront, maritime industrial, manufacturing, land use</t>
+        </is>
+      </c>
+      <c r="L31" s="5" t="inlineStr">
+        <is>
+          <t>https://legistar.council.nyc.gov/LegislationDetail.aspx?GUID=D8B4390B-0732-4EE5-9C0B-B46F6517FC9D&amp;ID=7861417</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="54" customHeight="1">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>MEDIUM PRIORITY</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>65</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>NYC Int 0058-2026</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Study of truck and delivery traffic generated by last-mile facilities</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>New York City Council</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>Committee on Transportation and Infrastructure</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>Referred to Committee</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="n">
+        <v>46051</v>
+      </c>
+      <c r="I32" s="3" t="n">
+        <v>111</v>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>Requires study of impacts from truck and delivery traffic generated by last-mile facilities on communities and infrastructure. Relevant to freight demand, warehouse impacts, truck routes, and port-linked distribution networks.</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>NYC, last mile, freight, truck traffic, logistics, infrastructure</t>
+        </is>
+      </c>
+      <c r="L32" s="5" t="inlineStr">
+        <is>
+          <t>https://legistar.council.nyc.gov/LegislationDetail.aspx?GUID=6B13C45C-0E7C-4B5C-B1AE-8C3777CBF012&amp;ID=7861424&amp;Options=&amp;Search=</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="54" customHeight="1">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>MEDIUM PRIORITY</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>65</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>NYC Int 0672-2026</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Reducing maximum time commercial vehicles may park</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>New York City Council</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>Committee on Transportation and Infrastructure</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>Referred to Committee</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="n">
+        <v>46065</v>
+      </c>
+      <c r="I33" s="3" t="n">
+        <v>97</v>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>Limits parking time for tractor-trailer combinations, tractors, truck trailers, and semi-trailers. Relevant to urban freight movement, curb management, commercial vehicle operations, and distribution impacts.</t>
+        </is>
+      </c>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>NYC, commercial vehicle, truck, freight, curb management, logistics</t>
+        </is>
+      </c>
+      <c r="L33" s="5" t="inlineStr">
+        <is>
+          <t>https://legistar.council.nyc.gov/LegislationDetail.aspx?GUID=F7281BB2-40E9-469F-B744-E51A0BCB656E&amp;ID=7878789</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="54" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>HIGH PRIORITY</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>NYC Int 0691-2026</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Commercial vehicle parking and truck routing enforcement training</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>New York City Council</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>Committee on Transportation and Infrastructure</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>Referred to Committee</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="n">
+        <v>46093</v>
+      </c>
+      <c r="I34" s="3" t="n">
+        <v>69</v>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>Requires police officer training on enforcement of commercial vehicle parking, stopping, standing, and truck routing rules. Relevant to freight mobility, truck route compliance, and community impacts near logistics corridors.</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>NYC, truck route, commercial vehicle, freight, logistics</t>
+        </is>
+      </c>
+      <c r="L34" s="5" t="inlineStr">
+        <is>
+          <t>https://legistar.council.nyc.gov/LegislationDetail.aspx?G=2FD004F1-D85B-4588-A648-0A736C77D6E3&amp;GUID=7A0DBA27-CE5F-4225-9B00-DE117444B008&amp;ID=7927486&amp;Options=&amp;Search=</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="54" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>HIGH PRIORITY</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>NYC Int 0819-2026</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Plan to increase freight rail operations and expand freight rail network</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>New York City Council</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>Committee on Economic Development</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>Committee</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="n">
+        <v>46128</v>
+      </c>
+      <c r="I35" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>Requires a plan to increase freight rail operations and expand the freight rail network. Relevant to modal shift, reducing truck dependency, intermodal freight planning, and Port of New York and New Jersey goods movement.</t>
+        </is>
+      </c>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t>NYC, freight rail, intermodal, logistics, supply chain, transportation</t>
+        </is>
+      </c>
+      <c r="L35" s="5" t="inlineStr">
+        <is>
+          <t>https://legistar.council.nyc.gov/LegislationDetail.aspx?GUID=83395820-53B2-44F2-BA8D-72F30065AE9E&amp;ID=7984575</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="54" customHeight="1">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>MEDIUM PRIORITY</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>NYC Res 0031-2026</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Calling on maritime importers to reduce truck traffic through marine vessels</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>New York City Council</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>New York City Council</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>Introduced</t>
+        </is>
+      </c>
+      <c r="H36" s="4" t="n">
+        <v>46051</v>
+      </c>
+      <c r="I36" s="3" t="n">
+        <v>111</v>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>Calls on top maritime importers to New York City ports to reduce truck traffic and use marine vessels for last-mile deliveries through Blue Highways-style service. Relevant to port cargo movement, truck congestion, emissions, and marine terminal use.</t>
+        </is>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>NYC, Port of New York and New Jersey, blue highways, marine vessels, cargo, freight</t>
+        </is>
+      </c>
+      <c r="L36" s="5" t="inlineStr">
+        <is>
+          <t>https://legistar.council.nyc.gov/LegislationDetail.aspx?From=RSS&amp;GUID=6DAA0B43-60D8-4A0E-8E6C-576C2FD1E101&amp;ID=7861438</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="54" customHeight="1">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>MEDIUM PRIORITY</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>55</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>NYC Int 1507-2025</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Truck route compliance and warehouse operators study</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>New York City Council</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Committee on Transportation and Infrastructure</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>Introduced</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="n">
+        <v>46008</v>
+      </c>
+      <c r="I37" s="3" t="n">
+        <v>154</v>
+      </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>Requires DOT to study and report on truck route compliance and warehouse operators. Relevant to port-linked warehousing, truck routes, community impacts, and urban freight planning.</t>
+        </is>
+      </c>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>NYC, truck route, warehouse, freight, logistics, distribution</t>
+        </is>
+      </c>
+      <c r="L37" s="5" t="inlineStr">
+        <is>
+          <t>https://legistar.council.nyc.gov/LegislationDetail.aspx?GUID=2F1E9BF6-D372-4D42-8A76-9882D25810F3&amp;ID=7785337</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L18"/>
-  <conditionalFormatting sqref="B2:B18">
+  <autoFilter ref="A1:L37"/>
+  <conditionalFormatting sqref="B2:B37">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
       <formula>80</formula>
     </cfRule>
@@ -1610,10 +2682,29 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId36"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId18"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId37"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1624,7 +2715,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1741,7 +2832,7 @@
         <v>45818</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
@@ -1797,7 +2888,7 @@
         <v>46149</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
@@ -1853,7 +2944,7 @@
         <v>46157</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
@@ -1867,7 +2958,7 @@
       </c>
       <c r="L4" s="5" t="inlineStr">
         <is>
-          <t>https://legislation.nysenate.gov/pdf/bills/2025/A11291</t>
+          <t>https://www.nysenate.gov/legislation/bills/2025/A11291</t>
         </is>
       </c>
     </row>
@@ -1909,7 +3000,7 @@
         <v>46097</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
@@ -1927,9 +3018,345 @@
         </is>
       </c>
     </row>
+    <row r="6" ht="54" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>HIGH PRIORITY</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>NJ A4236</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>High-growth STEM and transportation logistics workforce update</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey Assembly</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Labor</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Introduced</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>46076</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>86</v>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Updates high-growth industry and workforce language including transportation, logistics, and distribution. Relevant to workforce pathways that support port, freight, warehousing, and supply chain employers.</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey, workforce development, transportation, logistics, distribution</t>
+        </is>
+      </c>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>https://pub.njleg.state.nj.us/Bills/2026/A4500/4236_I1.HTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="54" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>HIGH PRIORITY</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>NJ S3593</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey Works Act pre-employment and work readiness training</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey Senate</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Labor</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Reported Committee</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>46083</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>79</v>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>Provides tax credits for approved pre-employment and work readiness training programs for in-demand jobs. Relevant to building workforce pipelines for logistics, port operations, and regional goods movement employers.</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey, workforce development, work readiness, logistics, training</t>
+        </is>
+      </c>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>https://pub.njleg.state.nj.us/Bills/2026/S4000/3593_S1.HTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="54" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>HIGH PRIORITY</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>NJ S3695</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Transportation Authority of New Jersey governance and transfer act</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey Senate</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Introduced</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>46077</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>Creates a statewide transportation authority structure and transfers certain transportation entities while preserving rules, bonding powers, employees, and operational obligations. Relevant as a New Jersey transportation governance and infrastructure oversight watch item.</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey, transportation authority, infrastructure, governance, operations, workforce</t>
+        </is>
+      </c>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>https://pub.njleg.state.nj.us/Bills/2026/S4000/3695_I1.HTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="54" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>HIGH PRIORITY</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>NJ S3790</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Transportation authority reporting and Port Authority-related oversight</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey Senate</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Introduced</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>46122</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>Requires reporting and oversight related to major transportation authorities and references the Port Authority of New York and New Jersey. Relevant to governance, accountability, workforce, and regional transportation policy monitoring.</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>New Jersey, PANYNJ, Port Authority, transportation authority, oversight, workforce</t>
+        </is>
+      </c>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>https://pub.njleg.state.nj.us/Bills/2026/S4000/3790_I1.PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="54" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>HIGH PRIORITY</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>NYC Int 0691-2026</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Commercial vehicle parking and truck routing enforcement training</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>New York City Council</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Committee on Transportation and Infrastructure</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Referred to Committee</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>46093</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>69</v>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>Requires police officer training on enforcement of commercial vehicle parking, stopping, standing, and truck routing rules. Relevant to freight mobility, truck route compliance, and community impacts near logistics corridors.</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>NYC, truck route, commercial vehicle, freight, logistics</t>
+        </is>
+      </c>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>https://legistar.council.nyc.gov/LegislationDetail.aspx?G=2FD004F1-D85B-4588-A648-0A736C77D6E3&amp;GUID=7A0DBA27-CE5F-4225-9B00-DE117444B008&amp;ID=7927486&amp;Options=&amp;Search=</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="54" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>HIGH PRIORITY</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>NYC Int 0819-2026</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Plan to increase freight rail operations and expand freight rail network</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>New York City Council</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Committee on Economic Development</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Committee</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>46128</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>Requires a plan to increase freight rail operations and expand the freight rail network. Relevant to modal shift, reducing truck dependency, intermodal freight planning, and Port of New York and New Jersey goods movement.</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>NYC, freight rail, intermodal, logistics, supply chain, transportation</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>https://legistar.council.nyc.gov/LegislationDetail.aspx?GUID=83395820-53B2-44F2-BA8D-72F30065AE9E&amp;ID=7984575</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L5"/>
-  <conditionalFormatting sqref="B2:B5">
+  <autoFilter ref="A1:L11"/>
+  <conditionalFormatting sqref="B2:B11">
     <cfRule type="cellIs" priority="1" operator="greaterThanOrEqual" dxfId="0">
       <formula>80</formula>
     </cfRule>
@@ -1946,10 +3373,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1960,7 +3393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2004,7 +3437,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="C2" s="3" t="inlineStr"/>
       <c r="D2" s="3" t="inlineStr"/>
@@ -2017,7 +3450,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="3" t="inlineStr"/>
@@ -2030,7 +3463,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="C4" s="3" t="inlineStr"/>
       <c r="D4" s="3" t="inlineStr"/>
@@ -2043,7 +3476,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
       <c r="D5" s="3" t="inlineStr"/>
@@ -2056,7 +3489,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>69.41</v>
+        <v>69.31</v>
       </c>
       <c r="C6" s="3" t="inlineStr"/>
       <c r="D6" s="3" t="inlineStr"/>
@@ -2078,10 +3511,10 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>65</v>
+        <v>61.67</v>
       </c>
     </row>
     <row r="9" ht="12" customHeight="1">
@@ -2104,14 +3537,14 @@
       <c r="B10" s="3" t="inlineStr"/>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Corporations, Authorities And Commissions</t>
+          <t>Commerce; Energy and Commerce</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>80</v>
+        <v>65</v>
       </c>
     </row>
     <row r="11" ht="12" customHeight="1">
@@ -2119,14 +3552,14 @@
       <c r="B11" s="3" t="inlineStr"/>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Environment and Public Works</t>
+          <t>Committee on Economic Development</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" ht="12" customHeight="1">
@@ -2134,14 +3567,14 @@
       <c r="B12" s="3" t="inlineStr"/>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>House Transportation and Infrastructure; Senate Commerce</t>
+          <t>Committee on Transportation and Infrastructure</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>80</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" ht="12" customHeight="1">
@@ -2149,14 +3582,14 @@
       <c r="B13" s="3" t="inlineStr"/>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Transportation</t>
+          <t>Committee on Zoning and Franchises</t>
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>76.67</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" ht="12" customHeight="1">
@@ -2164,14 +3597,14 @@
       <c r="B14" s="3" t="inlineStr"/>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Transportation and Infrastructure</t>
+          <t>Corporations, Authorities And Commissions</t>
         </is>
       </c>
       <c r="D14" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>60</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" ht="12" customHeight="1">
@@ -2179,7 +3612,7 @@
       <c r="B15" s="3" t="inlineStr"/>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Transportation and Infrastructure; Environment and Public Works</t>
+          <t>Environment and Public Works</t>
         </is>
       </c>
       <c r="D15" s="3" t="n">
@@ -2189,8 +3622,98 @@
         <v>70</v>
       </c>
     </row>
+    <row r="16" ht="12" customHeight="1">
+      <c r="A16" s="3" t="inlineStr"/>
+      <c r="B16" s="3" t="inlineStr"/>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>House Transportation and Infrastructure; Senate Commerce</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17" ht="12" customHeight="1">
+      <c r="A17" s="3" t="inlineStr"/>
+      <c r="B17" s="3" t="inlineStr"/>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Labor</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>86.67</v>
+      </c>
+    </row>
+    <row r="18" ht="12" customHeight="1">
+      <c r="A18" s="3" t="inlineStr"/>
+      <c r="B18" s="3" t="inlineStr"/>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>New York City Council</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="19" ht="12" customHeight="1">
+      <c r="A19" s="3" t="inlineStr"/>
+      <c r="B19" s="3" t="inlineStr"/>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>78.33</v>
+      </c>
+    </row>
+    <row r="20" ht="12" customHeight="1">
+      <c r="A20" s="3" t="inlineStr"/>
+      <c r="B20" s="3" t="inlineStr"/>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Transportation and Infrastructure</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="21" ht="12" customHeight="1">
+      <c r="A21" s="3" t="inlineStr"/>
+      <c r="B21" s="3" t="inlineStr"/>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Transportation and Infrastructure; Environment and Public Works</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>70</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E15"/>
+  <autoFilter ref="A1:E21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>